<commit_message>
new constraint type MININROW
</commit_message>
<xml_diff>
--- a/SEQUENCE_MODEL_DEFINITION_MANUAL.xlsx
+++ b/SEQUENCE_MODEL_DEFINITION_MANUAL.xlsx
@@ -1,16 +1,11 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="30228"/>
-  <workbookPr/>
-  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-    <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\4900063\Work\SCIENCE\papers\optimization_1\APP\"/>
-    </mc:Choice>
-  </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{775C51DD-7C97-43D1-B41D-F0E93264AC13}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="30326"/>
+  <workbookPr filterPrivacy="1"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{187A9599-A5CF-4AFB-A1CF-06D70BC1BE3A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="38280" yWindow="-120" windowWidth="38640" windowHeight="21120" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="40785" yWindow="2235" windowWidth="31770" windowHeight="16905" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="ATTRIBUTES" sheetId="1" r:id="rId1"/>
@@ -4351,6 +4346,7 @@
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
 </worksheet>
 </file>
 
@@ -4738,6 +4734,7 @@
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
   <headerFooter>
     <oddHeader>&amp;C&amp;G</oddHeader>
   </headerFooter>
@@ -6903,6 +6900,7 @@
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
 </worksheet>
 </file>
 

</xml_diff>